<commit_message>
adding UI functionality to Calendar component
added extra state and styling and validity checks to the Calendar component. Added alters to tell customer of errrors.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38836A4-DF96-49EC-9068-D8B8501999F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D987F59F-8DD2-4532-81DA-6CA30C4D2FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="121">
   <si>
     <t>Date</t>
   </si>
@@ -389,6 +389,21 @@
   </si>
   <si>
     <t>start of week format</t>
+  </si>
+  <si>
+    <t>react-big-calendar</t>
+  </si>
+  <si>
+    <t>onSeclectEvent</t>
+  </si>
+  <si>
+    <t>Calendar's onSelectEvent</t>
+  </si>
+  <si>
+    <t>calendar setup and localiser</t>
+  </si>
+  <si>
+    <t>starting code for calendar and localiser</t>
   </si>
 </sst>
 </file>
@@ -800,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1253,16 +1268,16 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>45996</v>
+        <v>45993</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1270,13 +1285,41 @@
         <v>45996</v>
       </c>
       <c r="B35" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>45996</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C36" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>45998</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1313,11 +1356,13 @@
     <hyperlink ref="C32" r:id="rId29" xr:uid="{F1C3C78B-B8E6-48A4-8F51-5148F47AE238}"/>
     <hyperlink ref="C31" r:id="rId30" xr:uid="{7D53FE41-D04E-4CFD-855A-40B65B7655E2}"/>
     <hyperlink ref="C33" r:id="rId31" xr:uid="{254DFCB9-A620-4255-A697-2CB786CA7CE3}"/>
-    <hyperlink ref="C34" r:id="rId32" xr:uid="{9199EC49-22AB-4322-AC33-4F2E57753EE3}"/>
-    <hyperlink ref="C35" r:id="rId33" xr:uid="{01609D78-3D3A-47F8-BF5A-5FF917290433}"/>
+    <hyperlink ref="C35" r:id="rId32" xr:uid="{9199EC49-22AB-4322-AC33-4F2E57753EE3}"/>
+    <hyperlink ref="C36" r:id="rId33" xr:uid="{01609D78-3D3A-47F8-BF5A-5FF917290433}"/>
+    <hyperlink ref="C37" r:id="rId34" xr:uid="{3606DB42-0C27-49DA-ACF9-27FB2D79623A}"/>
+    <hyperlink ref="C34" r:id="rId35" xr:uid="{255A3E96-C2D8-4932-B7F1-72D2BB7D9B98}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId34"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId36"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Calendar component extra functionality
Added extra frotnend functionality: different styling for draft and confirmed events. Cancel bookings. Check for overlapping bookings and prevent it occuring. Added a panel that displays event info on clicking the event. and is removed when the event is clicked again. Added functions for formatting the date and times of events in to nicer strings for UI.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D987F59F-8DD2-4532-81DA-6CA30C4D2FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C791BAAD-B5AD-428C-ADCE-7A71EB81A0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="127">
   <si>
     <t>Date</t>
   </si>
@@ -404,6 +404,24 @@
   </si>
   <si>
     <t>starting code for calendar and localiser</t>
+  </si>
+  <si>
+    <t>eventPropGetter</t>
+  </si>
+  <si>
+    <t>custom styling of Calendar events</t>
+  </si>
+  <si>
+    <t>toLocaleDateString()</t>
+  </si>
+  <si>
+    <t>mdn docs</t>
+  </si>
+  <si>
+    <t>method usage</t>
+  </si>
+  <si>
+    <t>toLocaleTimeString()</t>
   </si>
 </sst>
 </file>
@@ -815,7 +833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1320,6 +1338,48 @@
       </c>
       <c r="D37" s="3" t="s">
         <v>118</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
+        <v>45998</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
+        <v>45999</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="5">
+        <v>45999</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1360,9 +1420,12 @@
     <hyperlink ref="C36" r:id="rId33" xr:uid="{01609D78-3D3A-47F8-BF5A-5FF917290433}"/>
     <hyperlink ref="C37" r:id="rId34" xr:uid="{3606DB42-0C27-49DA-ACF9-27FB2D79623A}"/>
     <hyperlink ref="C34" r:id="rId35" xr:uid="{255A3E96-C2D8-4932-B7F1-72D2BB7D9B98}"/>
+    <hyperlink ref="C38" r:id="rId36" xr:uid="{0547D2F1-2A1F-4CE3-86EF-58E23F51E94A}"/>
+    <hyperlink ref="C39" r:id="rId37" xr:uid="{A68626F7-6347-4DAC-B7E4-420C7B476A2F}"/>
+    <hyperlink ref="C40" r:id="rId38" xr:uid="{CB9BD13E-9B50-44C5-82C4-024640EDF863}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId36"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId39"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
improvements to booking functionality UI
amended frontend and backend to prevent cancelling an appointment within 24 hours of start time. This required new functions on front end and backend and modified sql queries on backend and use of the postgres interval data type/function

Added extra styling in calendar comonent for bookings that are due to starft in less than 24 hours.

Chanhe dcalendar slots from 30 minute duration to 15 minute duration
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D8F3D7-FFDF-49C2-A2AF-44D8415290A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4082E4B-0927-4BCE-B21A-9F017BB3E267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="130">
   <si>
     <t>Date</t>
   </si>
@@ -422,6 +422,15 @@
   </si>
   <si>
     <t>toLocaleTimeString()</t>
+  </si>
+  <si>
+    <t>postgres interval</t>
+  </si>
+  <si>
+    <t>postgres tutorial</t>
+  </si>
+  <si>
+    <t>interval function</t>
   </si>
 </sst>
 </file>
@@ -1383,8 +1392,18 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="5"/>
-      <c r="C41" s="6"/>
+      <c r="A41" s="5">
+        <v>46033</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>129</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1427,9 +1446,10 @@
     <hyperlink ref="C38" r:id="rId36" xr:uid="{0547D2F1-2A1F-4CE3-86EF-58E23F51E94A}"/>
     <hyperlink ref="C39" r:id="rId37" xr:uid="{A68626F7-6347-4DAC-B7E4-420C7B476A2F}"/>
     <hyperlink ref="C40" r:id="rId38" xr:uid="{CB9BD13E-9B50-44C5-82C4-024640EDF863}"/>
+    <hyperlink ref="C41" r:id="rId39" xr:uid="{816ECC41-1389-44F8-9A20-42011A9E6079}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId39"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId40"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update to servber.io/webchat branch
copious changesand new code. full notes will be added on later updates
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903368B1-2000-4267-B6A4-E9A67AE6C956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143330AB-F02D-4EAA-9AFE-D1794CBD7CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
   <sheets>
     <sheet name="inspriation sources" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="146">
   <si>
     <t>Date</t>
   </si>
@@ -470,6 +470,15 @@
   </si>
   <si>
     <t>how to create socket.io middleware and ensure client  sends required auth token</t>
+  </si>
+  <si>
+    <t>socket.io data</t>
+  </si>
+  <si>
+    <t>adding data to socket object</t>
+  </si>
+  <si>
+    <t>stack overflow shows to use socket.data object to add data</t>
   </si>
 </sst>
 </file>
@@ -881,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1534,6 +1543,20 @@
       </c>
       <c r="D48" s="3" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="5">
+        <v>46063</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1585,9 +1608,10 @@
     <hyperlink ref="C46" r:id="rId44" xr:uid="{D1A2AF0B-0CA2-407A-B6B1-EA7B73E18591}"/>
     <hyperlink ref="C47" r:id="rId45" location="auth" xr:uid="{BC5DCA87-B939-4246-9E7B-C0D371B8B3B4}"/>
     <hyperlink ref="C48" r:id="rId46" location="sending-credentials" xr:uid="{ABE0F341-2A39-4173-9F0A-66003E4641B7}"/>
+    <hyperlink ref="C49" r:id="rId47" xr:uid="{2E62C5DE-3858-4683-89AA-22F59BF60F30}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId47"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId48"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
socket.io message DB persisence
added code to persist messages to DB. Added two new DB tables with constrainsts.  Added query logic in to the socket..on('chat_message') event in the server i.e. how the server responds when it receives a message from client's ChatWindow.  Too tired to add more notes. Need to get the ChatWondow component to fetch chst hostory on opening and also reformat appearance as per tsupervisor feedback
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143330AB-F02D-4EAA-9AFE-D1794CBD7CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9837EB9-1B91-492E-B5A3-2E2F9CEBA9FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="152">
   <si>
     <t>Date</t>
   </si>
@@ -479,6 +479,24 @@
   </si>
   <si>
     <t>stack overflow shows to use socket.data object to add data</t>
+  </si>
+  <si>
+    <t>postgres upsert</t>
+  </si>
+  <si>
+    <t>used in socket.io to reduce DB searches</t>
+  </si>
+  <si>
+    <t>10-17/2/26</t>
+  </si>
+  <si>
+    <t>socket.io + react webchat</t>
+  </si>
+  <si>
+    <t>webchat</t>
+  </si>
+  <si>
+    <t>codesistency on youtube</t>
   </si>
 </sst>
 </file>
@@ -890,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1557,6 +1575,34 @@
       </c>
       <c r="D49" s="3" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>46070</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -1609,9 +1655,11 @@
     <hyperlink ref="C47" r:id="rId45" location="auth" xr:uid="{BC5DCA87-B939-4246-9E7B-C0D371B8B3B4}"/>
     <hyperlink ref="C48" r:id="rId46" location="sending-credentials" xr:uid="{ABE0F341-2A39-4173-9F0A-66003E4641B7}"/>
     <hyperlink ref="C49" r:id="rId47" xr:uid="{2E62C5DE-3858-4683-89AA-22F59BF60F30}"/>
+    <hyperlink ref="C51" r:id="rId48" xr:uid="{F155139A-3434-4782-B615-64B486D351D1}"/>
+    <hyperlink ref="C50" r:id="rId49" xr:uid="{76697DBB-3F51-4C18-B8A6-8E781AB753A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId48"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId50"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
adding dissertation draft as work in progress
adding dissertation draft as work in progress
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9837EB9-1B91-492E-B5A3-2E2F9CEBA9FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5613477-F297-4AD4-85A7-A87F5B2DA9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
   <sheets>
     <sheet name="inspriation sources" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="155">
   <si>
     <t>Date</t>
   </si>
@@ -497,6 +497,15 @@
   </si>
   <si>
     <t>codesistency on youtube</t>
+  </si>
+  <si>
+    <t>referenced at</t>
+  </si>
+  <si>
+    <t>3.2.1</t>
+  </si>
+  <si>
+    <t>3.2.2</t>
   </si>
 </sst>
 </file>
@@ -908,17 +917,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="92.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="89.7109375" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="4"/>
+    <col min="5" max="5" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -931,8 +941,11 @@
       <c r="D1" s="3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>45931</v>
       </c>
@@ -943,7 +956,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>45932</v>
       </c>
@@ -953,8 +966,14 @@
       <c r="C3" s="6" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>45933</v>
       </c>
@@ -964,8 +983,14 @@
       <c r="C4" s="6" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F4" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>45934</v>
       </c>
@@ -975,8 +1000,14 @@
       <c r="C5" s="6" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F5" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>45935</v>
       </c>
@@ -986,8 +1017,14 @@
       <c r="C6" s="6" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>45936</v>
       </c>
@@ -997,8 +1034,14 @@
       <c r="C7" s="6" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>45937</v>
       </c>
@@ -1011,8 +1054,14 @@
       <c r="D8" s="3" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="E8" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>45938</v>
       </c>
@@ -1025,8 +1074,14 @@
       <c r="D9" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E9" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F9" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>45939</v>
       </c>
@@ -1039,8 +1094,14 @@
       <c r="D10" s="3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>45940</v>
       </c>
@@ -1053,8 +1114,14 @@
       <c r="D11" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F11" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>45941</v>
       </c>
@@ -1068,7 +1135,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>45942</v>
       </c>
@@ -1082,7 +1149,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>45943</v>
       </c>
@@ -1096,7 +1163,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>45944</v>
       </c>
@@ -1110,7 +1177,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>45945</v>
       </c>
@@ -1123,8 +1190,14 @@
       <c r="D16" s="3" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F16" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>45946</v>
       </c>
@@ -1138,7 +1211,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>45947</v>
       </c>
@@ -1152,7 +1225,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>45948</v>
       </c>
@@ -1166,7 +1239,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>45949</v>
       </c>
@@ -1180,7 +1253,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>45950</v>
       </c>
@@ -1194,7 +1267,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>45951</v>
       </c>
@@ -1208,7 +1281,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>45952</v>
       </c>
@@ -1222,7 +1295,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>45953</v>
       </c>
@@ -1236,7 +1309,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>45954</v>
       </c>
@@ -1250,7 +1323,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>45955</v>
       </c>
@@ -1264,7 +1337,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>45956</v>
       </c>
@@ -1278,7 +1351,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>45957</v>
       </c>
@@ -1291,8 +1364,14 @@
       <c r="D28" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>45958</v>
       </c>
@@ -1303,7 +1382,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>45963</v>
       </c>
@@ -1317,7 +1396,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>45971</v>
       </c>
@@ -1331,7 +1410,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>45973</v>
       </c>

</xml_diff>

<commit_message>
real-time message fiunctionality write up
most of the write up done.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64CBA12-9357-4C9B-8EC9-F00B6112B96C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C17C83-1FD8-4317-B7F5-707F31A74957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="166">
   <si>
     <t>Date</t>
   </si>
@@ -536,6 +536,9 @@
   </si>
   <si>
     <t xml:space="preserve">ref no </t>
+  </si>
+  <si>
+    <t>3.2.5</t>
   </si>
 </sst>
 </file>
@@ -1803,6 +1806,12 @@
       <c r="C45" s="6" t="s">
         <v>131</v>
       </c>
+      <c r="E45" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="4">
+        <v>39</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
@@ -1814,6 +1823,12 @@
       <c r="C46" s="6" t="s">
         <v>135</v>
       </c>
+      <c r="E46" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F46" s="4">
+        <v>40</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
@@ -1828,6 +1843,12 @@
       <c r="D47" s="3" t="s">
         <v>134</v>
       </c>
+      <c r="E47" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F47" s="4">
+        <v>41</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
@@ -1842,8 +1863,14 @@
       <c r="D48" s="3" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E48" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F48" s="4">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
         <v>46054</v>
       </c>
@@ -1856,8 +1883,14 @@
       <c r="D49" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F49" s="4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>46054</v>
       </c>
@@ -1870,8 +1903,14 @@
       <c r="D50" s="3" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E50" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F50" s="4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>46054</v>
       </c>
@@ -1884,8 +1923,14 @@
       <c r="D51" s="3" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F51" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
         <v>46063</v>
       </c>
@@ -1898,8 +1943,14 @@
       <c r="D52" s="3" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F52" s="4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>148</v>
       </c>
@@ -1912,8 +1963,14 @@
       <c r="D53" s="3" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F53" s="4">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>46070</v>
       </c>
@@ -1925,6 +1982,12 @@
       </c>
       <c r="D54" s="3" t="s">
         <v>147</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F54" s="4">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-write of chapter 3
re-write of chapter 3
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C17C83-1FD8-4317-B7F5-707F31A74957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D12A02-A3EA-4AAC-97F8-DFDF4DB149F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="169">
   <si>
     <t>Date</t>
   </si>
@@ -539,6 +539,15 @@
   </si>
   <si>
     <t>3.2.5</t>
+  </si>
+  <si>
+    <t>https://kitrum.com/blog/client-server-architecture-advantages-and-disadvantages/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/system-design/client-server-architecture-system-design/</t>
+  </si>
+  <si>
+    <t>https://medium.com/nerd-for-tech/client-server-architecture-explained-with-examples-diagrams-and-real-world-applications-407e9e04e2d1</t>
   </si>
 </sst>
 </file>
@@ -950,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -1988,6 +1997,21 @@
       </c>
       <c r="F54" s="4">
         <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C55" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C56" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C57" s="4" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dissertation extra info and new route handler to being re-auth
Rewrote and extended chapter 3 in dissertation. Began testing chapyter.

Also began trying to fix issue with losing user staus on frotnend when page has full refresh.  Saving current status and will create a new branch for this attempt.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D12A02-A3EA-4AAC-97F8-DFDF4DB149F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82539682-CFBF-4115-934D-BFA74536BB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="174">
   <si>
     <t>Date</t>
   </si>
@@ -548,6 +548,21 @@
   </si>
   <si>
     <t>https://medium.com/nerd-for-tech/client-server-architecture-explained-with-examples-diagrams-and-real-world-applications-407e9e04e2d1</t>
+  </si>
+  <si>
+    <t>ref for</t>
+  </si>
+  <si>
+    <t>user registration</t>
+  </si>
+  <si>
+    <t>tutor searching</t>
+  </si>
+  <si>
+    <t>lesson booking</t>
+  </si>
+  <si>
+    <t>real-time messaging</t>
   </si>
 </sst>
 </file>
@@ -959,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -967,10 +982,12 @@
     <col min="3" max="3" width="92.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="89.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="4"/>
+    <col min="6" max="6" width="9.140625" style="4"/>
+    <col min="7" max="7" width="19.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -989,8 +1006,11 @@
       <c r="F1" s="4" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>45931</v>
       </c>
@@ -1007,7 +1027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>45931</v>
       </c>
@@ -1024,7 +1044,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>45932</v>
       </c>
@@ -1040,8 +1060,11 @@
       <c r="F4" s="4">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>45933</v>
       </c>
@@ -1057,8 +1080,11 @@
       <c r="F5" s="4">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>45934</v>
       </c>
@@ -1074,8 +1100,11 @@
       <c r="F6" s="4">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>45935</v>
       </c>
@@ -1091,8 +1120,11 @@
       <c r="F7" s="4">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>45936</v>
       </c>
@@ -1108,8 +1140,11 @@
       <c r="F8" s="4">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>45937</v>
       </c>
@@ -1128,8 +1163,11 @@
       <c r="F9" s="4">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="G9" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>45938</v>
       </c>
@@ -1148,8 +1186,11 @@
       <c r="F10" s="4">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G10" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>45939</v>
       </c>
@@ -1168,8 +1209,11 @@
       <c r="F11" s="4">
         <v>25</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>45940</v>
       </c>
@@ -1188,8 +1232,11 @@
       <c r="F12" s="4">
         <v>26</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>45941</v>
       </c>
@@ -1209,7 +1256,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>45942</v>
       </c>
@@ -1229,7 +1276,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>45943</v>
       </c>
@@ -1249,7 +1296,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>45944</v>
       </c>
@@ -1565,7 +1612,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>45971</v>
       </c>
@@ -1584,8 +1631,11 @@
       <c r="F33" s="4">
         <v>27</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>45973</v>
       </c>
@@ -1604,8 +1654,11 @@
       <c r="F34" s="4">
         <v>28</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>45993</v>
       </c>
@@ -1624,8 +1677,11 @@
       <c r="F35" s="4">
         <v>29</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>45993</v>
       </c>
@@ -1644,8 +1700,11 @@
       <c r="F36" s="4">
         <v>30</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>45993</v>
       </c>
@@ -1664,8 +1723,11 @@
       <c r="F37" s="4">
         <v>31</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>45996</v>
       </c>
@@ -1684,8 +1746,11 @@
       <c r="F38" s="4">
         <v>32</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>45996</v>
       </c>
@@ -1704,8 +1769,11 @@
       <c r="F39" s="4">
         <v>33</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>45998</v>
       </c>
@@ -1724,8 +1792,11 @@
       <c r="F40" s="4">
         <v>34</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>45998</v>
       </c>
@@ -1744,8 +1815,11 @@
       <c r="F41" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>45999</v>
       </c>
@@ -1764,8 +1838,11 @@
       <c r="F42" s="4">
         <v>36</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>45999</v>
       </c>
@@ -1784,8 +1861,11 @@
       <c r="F43" s="4">
         <v>37</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>46033</v>
       </c>
@@ -1804,8 +1884,11 @@
       <c r="F44" s="4">
         <v>38</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
         <v>45677</v>
       </c>
@@ -1821,8 +1904,11 @@
       <c r="F45" s="4">
         <v>39</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
         <v>46048</v>
       </c>
@@ -1838,8 +1924,11 @@
       <c r="F46" s="4">
         <v>40</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
         <v>46053</v>
       </c>
@@ -1858,8 +1947,11 @@
       <c r="F47" s="4">
         <v>41</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
         <v>46053</v>
       </c>
@@ -1878,8 +1970,11 @@
       <c r="F48" s="4">
         <v>42</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
         <v>46054</v>
       </c>
@@ -1898,8 +1993,11 @@
       <c r="F49" s="4">
         <v>43</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>46054</v>
       </c>
@@ -1918,8 +2016,11 @@
       <c r="F50" s="4">
         <v>44</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>46054</v>
       </c>
@@ -1938,8 +2039,11 @@
       <c r="F51" s="4">
         <v>45</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
         <v>46063</v>
       </c>
@@ -1958,8 +2062,11 @@
       <c r="F52" s="4">
         <v>46</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>148</v>
       </c>
@@ -1978,8 +2085,11 @@
       <c r="F53" s="4">
         <v>47</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>46070</v>
       </c>
@@ -1998,18 +2108,30 @@
       <c r="F54" s="4">
         <v>48</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46096</v>
+      </c>
       <c r="C55" s="4" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>46096</v>
+      </c>
       <c r="C56" s="4" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>46096</v>
+      </c>
       <c r="C57" s="4" t="s">
         <v>168</v>
       </c>

</xml_diff>

<commit_message>
Chapter 2 of dissertaion
Began chapter 2 and also improved UI responsiveness.

Login user form has the app logo set to rounded-full so its radius if fully circular.

Home page had ?. accessors on user first_name and last_name for rendering.

FindTutor page's search inputs given whote background.

Contact page's 'send message' button given cursor pointer.

about page given links in text to the findTutor page and Register page.

RootLayout's encompassing div given salte-100 background

FocusedTutorCard component 'Levels' <p> tag given 'wrap-anywhere' classname so that its text does not run off the card's boundary.

LogOut button's  logout function now forces navigation to the 'about' page after logout by using useNavigate() hook.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB44EF62-3773-4DE6-B171-14005A4E8B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BDA364-725D-4BBB-A47E-56ADC62D6FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="181">
   <si>
     <t>Date</t>
   </si>
@@ -575,6 +575,15 @@
   </si>
   <si>
     <t>zod on server custom validation and handling errors</t>
+  </si>
+  <si>
+    <t>react router</t>
+  </si>
+  <si>
+    <t>navlink</t>
+  </si>
+  <si>
+    <t>NavLinkRenderProps</t>
   </si>
 </sst>
 </file>
@@ -986,7 +995,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F90D4E2F-31CB-4504-B764-69927272A7DB}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -2174,6 +2183,20 @@
       </c>
       <c r="D59" s="3" t="s">
         <v>177</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2233,9 +2256,10 @@
     <hyperlink ref="C31" r:id="rId52" xr:uid="{FDF38111-75A7-4BE4-AD7C-E239437BE1BB}"/>
     <hyperlink ref="C58" r:id="rId53" xr:uid="{4BCBB930-2600-4BD0-A0FF-9565BB17D6B7}"/>
     <hyperlink ref="C59" r:id="rId54" xr:uid="{68912D8D-3E16-4512-951C-42E1A4EE1252}"/>
+    <hyperlink ref="C60" r:id="rId55" xr:uid="{E2B7A8BA-660B-4E6E-A449-BE8D06318890}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId55"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId56"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
dissertaion final draft before sub mssion
final draft before submission.
</commit_message>
<xml_diff>
--- a/docs/resource log.xlsx
+++ b/docs/resource log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\halog\Desktop\Music_Tutor_Project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BDA364-725D-4BBB-A47E-56ADC62D6FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E16CBFC-BFA5-41FC-B25B-B48AAB80C477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{41780912-9485-457E-8E39-EF1EA0B82C48}"/>
   </bookViews>
@@ -517,9 +517,6 @@
     <t>basic walkthrough</t>
   </si>
   <si>
-    <t>react</t>
-  </si>
-  <si>
     <t>anson dev</t>
   </si>
   <si>
@@ -584,6 +581,9 @@
   </si>
   <si>
     <t>NavLinkRenderProps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">express  </t>
   </si>
 </sst>
 </file>
@@ -1025,10 +1025,10 @@
         <v>152</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1036,10 +1036,10 @@
         <v>45931</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>159</v>
       </c>
       <c r="E2" s="4">
         <v>3.1</v>
@@ -1082,7 +1082,7 @@
         <v>18</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1102,7 +1102,7 @@
         <v>19</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1122,7 +1122,7 @@
         <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1142,7 +1142,7 @@
         <v>21</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1162,7 +1162,7 @@
         <v>22</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1185,7 +1185,7 @@
         <v>23</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="105" x14ac:dyDescent="0.25">
@@ -1208,7 +1208,7 @@
         <v>24</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -1231,7 +1231,7 @@
         <v>25</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1254,7 +1254,7 @@
         <v>26</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1348,7 +1348,7 @@
         <v>101</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E17" s="4">
         <v>3.1</v>
@@ -1604,13 +1604,13 @@
         <v>45957</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>162</v>
       </c>
       <c r="E31" s="4">
         <v>3.1</v>
@@ -1653,7 +1653,7 @@
         <v>27</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1676,7 +1676,7 @@
         <v>28</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1699,7 +1699,7 @@
         <v>29</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1722,7 +1722,7 @@
         <v>30</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1745,7 +1745,7 @@
         <v>31</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -1768,7 +1768,7 @@
         <v>32</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1791,7 +1791,7 @@
         <v>33</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -1814,7 +1814,7 @@
         <v>34</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1837,7 +1837,7 @@
         <v>35</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -1860,7 +1860,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1883,7 +1883,7 @@
         <v>37</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1906,7 +1906,7 @@
         <v>38</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -1920,13 +1920,13 @@
         <v>131</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F45" s="4">
         <v>39</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -1940,13 +1940,13 @@
         <v>135</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F46" s="4">
         <v>40</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -1963,13 +1963,13 @@
         <v>134</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F47" s="4">
         <v>41</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -1986,13 +1986,13 @@
         <v>133</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F48" s="4">
         <v>42</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -2009,13 +2009,13 @@
         <v>138</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F49" s="4">
         <v>43</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -2032,13 +2032,13 @@
         <v>140</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F50" s="4">
         <v>44</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -2055,13 +2055,13 @@
         <v>142</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F51" s="4">
         <v>45</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -2078,13 +2078,13 @@
         <v>145</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F52" s="4">
         <v>46</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -2101,13 +2101,13 @@
         <v>151</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F53" s="4">
         <v>47</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -2124,13 +2124,13 @@
         <v>147</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F54" s="4">
         <v>48</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -2138,7 +2138,7 @@
         <v>46096</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -2146,7 +2146,7 @@
         <v>46096</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -2154,7 +2154,7 @@
         <v>46096</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -2162,13 +2162,13 @@
         <v>46124</v>
       </c>
       <c r="B58" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="C58" s="6" t="s">
-        <v>175</v>
-      </c>
       <c r="D58" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
@@ -2176,13 +2176,13 @@
         <v>46124</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C59" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D59" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -2190,13 +2190,13 @@
         <v>46133</v>
       </c>
       <c r="B60" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C60" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="C60" s="6" t="s">
+      <c r="D60" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>